<commit_message>
modificacion de carta gantt
</commit_message>
<xml_diff>
--- a/Documentación/Diagrama de Gantt ágil1.xlsx
+++ b/Documentación/Diagrama de Gantt ágil1.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB9845E8-BC15-40B7-983A-3D8DE6AA64EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81046480-0CD3-4571-9198-1819F0E0DFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="415" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,28 +32,19 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
       <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
@@ -209,7 +200,7 @@
     <numFmt numFmtId="167" formatCode="d"/>
     <numFmt numFmtId="168" formatCode="#,##0_ ;\-#,##0\ "/>
   </numFmts>
-  <fonts count="46" x14ac:knownFonts="1">
+  <fonts count="47" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -534,6 +525,14 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1502,25 +1501,23 @@
     <xf numFmtId="14" fontId="20" fillId="10" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1530,6 +1527,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1544,22 +1556,9 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="46" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="20% - Énfasis1" xfId="28" builtinId="30" customBuiltin="1"/>
@@ -1614,6 +1613,24 @@
     <cellStyle name="zHiddenText" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
   <dxfs count="62">
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1681,24 +1698,6 @@
         <right/>
         <top/>
         <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -2104,39 +2103,6 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2278,6 +2244,39 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="1" tint="0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2795,7 +2794,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DD82988E-1813-40AE-BDE7-9F0200A703CB}" name="Hitos4352" displayName="Hitos4352" ref="B9:G36" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DD82988E-1813-40AE-BDE7-9F0200A703CB}" name="Hitos4352" displayName="Hitos4352" ref="B9:G36" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2805,12 +2804,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{619BF8F6-D0F1-41AD-871D-FE0240C45A93}" name="Descripción del hito" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{39BD914E-FB02-4352-846C-6D59624DC0B0}" name="Categoría" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{D274194F-BCA0-44F3-84B2-217254EE241C}" name="Asignado a" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{8385BC6F-56EE-4363-A106-8DB0A1E4EF5A}" name="Progreso" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{02926609-7B93-4B6F-BE96-92EC7A949E4B}" name="Inicio" dataDxfId="42" dataCellStyle="Fecha"/>
-    <tableColumn id="6" xr3:uid="{8FF9BE8E-04B7-4B39-AC27-D2E534204BC3}" name="Días" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{619BF8F6-D0F1-41AD-871D-FE0240C45A93}" name="Descripción del hito" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{39BD914E-FB02-4352-846C-6D59624DC0B0}" name="Categoría" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{D274194F-BCA0-44F3-84B2-217254EE241C}" name="Asignado a" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{8385BC6F-56EE-4363-A106-8DB0A1E4EF5A}" name="Progreso" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{02926609-7B93-4B6F-BE96-92EC7A949E4B}" name="Inicio" dataDxfId="37" dataCellStyle="Fecha"/>
+    <tableColumn id="6" xr3:uid="{8FF9BE8E-04B7-4B39-AC27-D2E534204BC3}" name="Días" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="ListaTareasPendientes" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -2822,7 +2821,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0EDB95CA-98FE-4198-8801-690B9B480FDF}" name="Hitos435" displayName="Hitos435" ref="B9:G36" totalsRowShown="0" headerRowDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0EDB95CA-98FE-4198-8801-690B9B480FDF}" name="Hitos435" displayName="Hitos435" ref="B9:G36" totalsRowShown="0" headerRowDxfId="35">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2832,9 +2831,9 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6E47A83D-ACD7-4EB6-9B84-5195E813945E}" name="Descripción del hito" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{529EEF64-D037-4ACF-8CA4-0C10FE2D1FBB}" name="Categoría" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{711D01BA-2785-403A-9636-CCC7E2ADA584}" name="Asignado a" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{6E47A83D-ACD7-4EB6-9B84-5195E813945E}" name="Descripción del hito" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{529EEF64-D037-4ACF-8CA4-0C10FE2D1FBB}" name="Categoría" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{711D01BA-2785-403A-9636-CCC7E2ADA584}" name="Asignado a" dataDxfId="32"/>
     <tableColumn id="4" xr3:uid="{62B00BEF-16BE-4692-B5E2-F287F680F2C1}" name="Progreso"/>
     <tableColumn id="5" xr3:uid="{D6D72902-F68F-4E59-A714-AFFF520C647A}" name="Inicio" dataCellStyle="Fecha"/>
     <tableColumn id="6" xr3:uid="{93E698DE-286F-49ED-AA20-D0C843671DE8}" name="Días"/>
@@ -2849,7 +2848,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{876EA49D-634E-482B-8173-880F7B761E2C}" name="Hitos43524" displayName="Hitos43524" ref="B9:G23" totalsRowShown="0" headerRowDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{876EA49D-634E-482B-8173-880F7B761E2C}" name="Hitos43524" displayName="Hitos43524" ref="B9:G23" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="B9:G23" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2859,11 +2858,11 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0971B905-713A-4980-8BBC-DF959C2E61F9}" name="Descripción del hito" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{4492A0B8-068F-4002-9E8D-E1F5FED367F0}" name="Categoría" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{DF1A764E-7050-4528-B7F9-B6AB99372146}" name="Asignado a" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{0971B905-713A-4980-8BBC-DF959C2E61F9}" name="Descripción del hito" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{4492A0B8-068F-4002-9E8D-E1F5FED367F0}" name="Categoría" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{DF1A764E-7050-4528-B7F9-B6AB99372146}" name="Asignado a" dataDxfId="45"/>
     <tableColumn id="4" xr3:uid="{47C54592-75B0-4C70-BBF8-0F40483670E9}" name="Progreso"/>
-    <tableColumn id="5" xr3:uid="{663FB5E0-7616-4EA5-B56A-FF069E2E07D7}" name="Inicio" dataDxfId="32" dataCellStyle="Fecha">
+    <tableColumn id="5" xr3:uid="{663FB5E0-7616-4EA5-B56A-FF069E2E07D7}" name="Inicio" dataDxfId="44" dataCellStyle="Fecha">
       <calculatedColumnFormula>TODAY()-35</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{3B766962-C06F-4E12-BE91-12AB93439874}" name="Días"/>
@@ -3158,11 +3157,11 @@
     <row r="2" spans="1:13" ht="50.1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="7"/>
       <c r="B2" s="96"/>
-      <c r="C2" s="123" t="s">
+      <c r="C2" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="123"/>
-      <c r="E2" s="123"/>
+      <c r="D2" s="133"/>
+      <c r="E2" s="133"/>
       <c r="F2" s="96"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
@@ -3190,11 +3189,11 @@
     <row r="4" spans="1:13" s="8" customFormat="1" ht="67.2" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="7"/>
       <c r="B4" s="91"/>
-      <c r="C4" s="124" t="s">
+      <c r="C4" s="134" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="124"/>
-      <c r="E4" s="124"/>
+      <c r="D4" s="134"/>
+      <c r="E4" s="134"/>
       <c r="F4" s="91"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
@@ -3207,11 +3206,11 @@
     <row r="5" spans="1:13" s="8" customFormat="1" ht="67.2" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="7"/>
       <c r="B5" s="91"/>
-      <c r="C5" s="124" t="s">
+      <c r="C5" s="134" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="124"/>
-      <c r="E5" s="124"/>
+      <c r="D5" s="134"/>
+      <c r="E5" s="134"/>
       <c r="F5" s="91"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
@@ -3325,27 +3324,27 @@
     <row r="1" spans="1:68" ht="25.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:68" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10"/>
-      <c r="B2" s="127" t="s">
+      <c r="B2" s="135" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="127"/>
-      <c r="D2" s="127"/>
-      <c r="E2" s="127"/>
-      <c r="F2" s="127"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="128"/>
-      <c r="K2" s="128"/>
-      <c r="L2" s="128"/>
-      <c r="M2" s="128"/>
-      <c r="N2" s="128"/>
-      <c r="O2" s="129"/>
-      <c r="P2" s="129"/>
-      <c r="Q2" s="129"/>
-      <c r="R2" s="129"/>
-      <c r="S2" s="129"/>
-      <c r="T2" s="129"/>
+      <c r="C2" s="135"/>
+      <c r="D2" s="135"/>
+      <c r="E2" s="135"/>
+      <c r="F2" s="135"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="135"/>
+      <c r="I2" s="136"/>
+      <c r="J2" s="136"/>
+      <c r="K2" s="136"/>
+      <c r="L2" s="136"/>
+      <c r="M2" s="136"/>
+      <c r="N2" s="136"/>
+      <c r="O2" s="137"/>
+      <c r="P2" s="137"/>
+      <c r="Q2" s="137"/>
+      <c r="R2" s="137"/>
+      <c r="S2" s="137"/>
+      <c r="T2" s="137"/>
       <c r="U2" s="60"/>
       <c r="V2" s="60"/>
       <c r="W2" s="60"/>
@@ -3469,7 +3468,7 @@
       </c>
       <c r="C6" s="73" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Hitos4352[Inicio])=0,TODAY(),B11(Hitos4352[Inicio])),TODAY())</f>
-        <v>46133</v>
+        <v>46141</v>
       </c>
       <c r="D6" s="73"/>
       <c r="E6" s="68"/>
@@ -3488,7 +3487,7 @@
       <c r="O6" s="83"/>
       <c r="P6" s="83" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>mayo</v>
       </c>
       <c r="Q6" s="83"/>
       <c r="R6" s="83"/>
@@ -3498,7 +3497,7 @@
       <c r="V6" s="83"/>
       <c r="W6" s="83" t="str">
         <f ca="1">IF(OR(TEXT(W7,"mmmm")=P6,TEXT(W7,"mmmm")=I6),"",TEXT(W7,"mmmm"))</f>
-        <v>mayo</v>
+        <v/>
       </c>
       <c r="X6" s="83"/>
       <c r="Y6" s="83"/>
@@ -3528,7 +3527,7 @@
       <c r="AQ6" s="83"/>
       <c r="AR6" s="83" t="str">
         <f ca="1">IF(OR(TEXT(AR7,"mmmm")=AK6,TEXT(AR7,"mmmm")=AD6,TEXT(AR7,"mmmm")=W6,TEXT(AR7,"mmmm")=P6),"",TEXT(AR7,"mmmm"))</f>
-        <v/>
+        <v>junio</v>
       </c>
       <c r="AS6" s="83"/>
       <c r="AT6" s="83"/>
@@ -3538,7 +3537,7 @@
       <c r="AX6" s="84"/>
       <c r="AY6" s="84" t="str">
         <f ca="1">IF(OR(TEXT(AY7,"mmmm")=AR6,TEXT(AY7,"mmmm")=AK6,TEXT(AY7,"mmmm")=AD6,TEXT(AY7,"mmmm")=W6),"",TEXT(AY7,"mmmm"))</f>
-        <v>junio</v>
+        <v/>
       </c>
       <c r="AZ6" s="84"/>
       <c r="BA6" s="84"/>
@@ -3572,227 +3571,227 @@
       <c r="H7" s="75"/>
       <c r="I7" s="107">
         <f ca="1">IFERROR(Inicio_del_proyecto+Incremento_de_desplazamiento,TODAY())</f>
-        <v>46134</v>
+        <v>46142</v>
       </c>
       <c r="J7" s="108">
         <f ca="1">I7+1</f>
-        <v>46135</v>
+        <v>46143</v>
       </c>
       <c r="K7" s="108">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46136</v>
+        <v>46144</v>
       </c>
       <c r="L7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46137</v>
+        <v>46145</v>
       </c>
       <c r="M7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46138</v>
+        <v>46146</v>
       </c>
       <c r="N7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="O7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="P7" s="108">
         <f ca="1">O7+1</f>
-        <v>46141</v>
+        <v>46149</v>
       </c>
       <c r="Q7" s="108">
         <f ca="1">P7+1</f>
-        <v>46142</v>
+        <v>46150</v>
       </c>
       <c r="R7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46143</v>
+        <v>46151</v>
       </c>
       <c r="S7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46144</v>
+        <v>46152</v>
       </c>
       <c r="T7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46145</v>
+        <v>46153</v>
       </c>
       <c r="U7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="V7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46147</v>
+        <v>46155</v>
       </c>
       <c r="W7" s="108">
         <f ca="1">V7+1</f>
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="X7" s="108">
         <f ca="1">W7+1</f>
-        <v>46149</v>
+        <v>46157</v>
       </c>
       <c r="Y7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46150</v>
+        <v>46158</v>
       </c>
       <c r="Z7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46151</v>
+        <v>46159</v>
       </c>
       <c r="AA7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46152</v>
+        <v>46160</v>
       </c>
       <c r="AB7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46153</v>
+        <v>46161</v>
       </c>
       <c r="AC7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46154</v>
+        <v>46162</v>
       </c>
       <c r="AD7" s="108">
         <f ca="1">AC7+1</f>
-        <v>46155</v>
+        <v>46163</v>
       </c>
       <c r="AE7" s="108">
         <f ca="1">AD7+1</f>
-        <v>46156</v>
+        <v>46164</v>
       </c>
       <c r="AF7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46157</v>
+        <v>46165</v>
       </c>
       <c r="AG7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46158</v>
+        <v>46166</v>
       </c>
       <c r="AH7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46159</v>
+        <v>46167</v>
       </c>
       <c r="AI7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46160</v>
+        <v>46168</v>
       </c>
       <c r="AJ7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46161</v>
+        <v>46169</v>
       </c>
       <c r="AK7" s="108">
         <f ca="1">AJ7+1</f>
-        <v>46162</v>
+        <v>46170</v>
       </c>
       <c r="AL7" s="108">
         <f ca="1">AK7+1</f>
-        <v>46163</v>
+        <v>46171</v>
       </c>
       <c r="AM7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46164</v>
+        <v>46172</v>
       </c>
       <c r="AN7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46165</v>
+        <v>46173</v>
       </c>
       <c r="AO7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46166</v>
+        <v>46174</v>
       </c>
       <c r="AP7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46167</v>
+        <v>46175</v>
       </c>
       <c r="AQ7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46168</v>
+        <v>46176</v>
       </c>
       <c r="AR7" s="108">
         <f ca="1">AQ7+1</f>
-        <v>46169</v>
+        <v>46177</v>
       </c>
       <c r="AS7" s="108">
         <f ca="1">AR7+1</f>
-        <v>46170</v>
+        <v>46178</v>
       </c>
       <c r="AT7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46171</v>
+        <v>46179</v>
       </c>
       <c r="AU7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46172</v>
+        <v>46180</v>
       </c>
       <c r="AV7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46173</v>
+        <v>46181</v>
       </c>
       <c r="AW7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="AX7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AY7" s="108">
         <f ca="1">AX7+1</f>
-        <v>46176</v>
+        <v>46184</v>
       </c>
       <c r="AZ7" s="108">
         <f ca="1">AY7+1</f>
-        <v>46177</v>
+        <v>46185</v>
       </c>
       <c r="BA7" s="108">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46178</v>
+        <v>46186</v>
       </c>
       <c r="BB7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46179</v>
+        <v>46187</v>
       </c>
       <c r="BC7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46180</v>
+        <v>46188</v>
       </c>
       <c r="BD7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46181</v>
+        <v>46189</v>
       </c>
       <c r="BE7" s="109">
         <f t="shared" ca="1" si="1"/>
-        <v>46182</v>
+        <v>46190</v>
       </c>
       <c r="BF7" s="108">
         <f ca="1">BE7+1</f>
-        <v>46183</v>
+        <v>46191</v>
       </c>
       <c r="BG7" s="108">
         <f ca="1">BF7+1</f>
-        <v>46184</v>
+        <v>46192</v>
       </c>
       <c r="BH7" s="108">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46185</v>
+        <v>46193</v>
       </c>
       <c r="BI7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46186</v>
+        <v>46194</v>
       </c>
       <c r="BJ7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46187</v>
+        <v>46195</v>
       </c>
       <c r="BK7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46188</v>
+        <v>46196</v>
       </c>
       <c r="BL7" s="109">
         <f t="shared" ca="1" si="2"/>
-        <v>46189</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3884,27 +3883,27 @@
       <c r="H9" s="80"/>
       <c r="I9" s="89" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="J9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="K9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="L9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="M9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="N9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="O9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3912,27 +3911,27 @@
       </c>
       <c r="P9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="Q9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="R9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="S9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="T9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="U9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="V9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3940,27 +3939,27 @@
       </c>
       <c r="W9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="X9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="Y9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="Z9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AA9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AB9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AC9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3968,27 +3967,27 @@
       </c>
       <c r="AD9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AE9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AF9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AG9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AH9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AI9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AJ9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3996,27 +3995,27 @@
       </c>
       <c r="AK9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AL9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AM9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AN9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AO9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AP9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AQ9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -4024,27 +4023,27 @@
       </c>
       <c r="AR9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AS9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AT9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AU9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AV9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AW9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AX9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -4052,27 +4051,27 @@
       </c>
       <c r="AY9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AZ9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="BA9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="BB9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="BC9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="BD9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="BE9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -4080,27 +4079,27 @@
       </c>
       <c r="BF9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="BG9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="BH9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="BI9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="BJ9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="BK9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="BL9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -4424,7 +4423,7 @@
       </c>
       <c r="F12" s="55">
         <f ca="1">TODAY()</f>
-        <v>46133</v>
+        <v>46141</v>
       </c>
       <c r="G12" s="56">
         <v>3</v>
@@ -4667,7 +4666,7 @@
       <c r="E13" s="54"/>
       <c r="F13" s="55">
         <f ca="1">TODAY()+5</f>
-        <v>46138</v>
+        <v>46146</v>
       </c>
       <c r="G13" s="56">
         <v>1</v>
@@ -4912,7 +4911,7 @@
       </c>
       <c r="F14" s="55">
         <f ca="1">F12-3</f>
-        <v>46130</v>
+        <v>46138</v>
       </c>
       <c r="G14" s="56">
         <v>10</v>
@@ -5155,7 +5154,7 @@
       <c r="E15" s="54"/>
       <c r="F15" s="55">
         <f ca="1">F12+20</f>
-        <v>46153</v>
+        <v>46161</v>
       </c>
       <c r="G15" s="56">
         <v>1</v>
@@ -5400,7 +5399,7 @@
       </c>
       <c r="F16" s="55">
         <f ca="1">F12+6</f>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="G16" s="56">
         <v>6</v>
@@ -5881,7 +5880,7 @@
       </c>
       <c r="F18" s="55">
         <f ca="1">F12+6</f>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="G18" s="56">
         <v>13</v>
@@ -6126,7 +6125,7 @@
       </c>
       <c r="F19" s="55">
         <f ca="1">F18+2</f>
-        <v>46141</v>
+        <v>46149</v>
       </c>
       <c r="G19" s="56">
         <v>9</v>
@@ -6371,7 +6370,7 @@
       </c>
       <c r="F20" s="55">
         <f ca="1">F19+5</f>
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="G20" s="56">
         <v>11</v>
@@ -6614,7 +6613,7 @@
       <c r="E21" s="54"/>
       <c r="F21" s="55">
         <f ca="1">F20+2</f>
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="G21" s="56">
         <v>1</v>
@@ -6855,7 +6854,7 @@
       <c r="E22" s="54"/>
       <c r="F22" s="55">
         <f ca="1">F21+1</f>
-        <v>46149</v>
+        <v>46157</v>
       </c>
       <c r="G22" s="56">
         <v>24</v>
@@ -7334,7 +7333,7 @@
       <c r="E24" s="54"/>
       <c r="F24" s="55">
         <f ca="1">F12+15</f>
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="G24" s="56">
         <v>4</v>
@@ -7577,7 +7576,7 @@
       <c r="E25" s="54"/>
       <c r="F25" s="55">
         <f ca="1">F24+3</f>
-        <v>46151</v>
+        <v>46159</v>
       </c>
       <c r="G25" s="56">
         <v>14</v>
@@ -7820,7 +7819,7 @@
       <c r="E26" s="54"/>
       <c r="F26" s="55">
         <f ca="1">F25+15</f>
-        <v>46166</v>
+        <v>46174</v>
       </c>
       <c r="G26" s="56">
         <v>6</v>
@@ -8063,7 +8062,7 @@
       <c r="E27" s="54"/>
       <c r="F27" s="55">
         <f ca="1">F21+22</f>
-        <v>46170</v>
+        <v>46178</v>
       </c>
       <c r="G27" s="56">
         <v>3</v>
@@ -8306,7 +8305,7 @@
       <c r="E28" s="54"/>
       <c r="F28" s="55">
         <f ca="1">F16</f>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="G28" s="56">
         <v>19</v>
@@ -8783,7 +8782,7 @@
       <c r="E30" s="54"/>
       <c r="F30" s="55">
         <f ca="1">F27+3</f>
-        <v>46173</v>
+        <v>46181</v>
       </c>
       <c r="G30" s="56">
         <v>15</v>
@@ -9024,7 +9023,7 @@
       <c r="E31" s="54"/>
       <c r="F31" s="55">
         <f ca="1">F30+14</f>
-        <v>46187</v>
+        <v>46195</v>
       </c>
       <c r="G31" s="56">
         <v>5</v>
@@ -9267,7 +9266,7 @@
       <c r="E32" s="54"/>
       <c r="F32" s="55">
         <f ca="1">F31+42</f>
-        <v>46229</v>
+        <v>46237</v>
       </c>
       <c r="G32" s="56">
         <v>1</v>
@@ -10484,27 +10483,27 @@
     <row r="1" spans="1:68" ht="25.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:68" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10"/>
-      <c r="B2" s="133" t="s">
+      <c r="B2" s="138" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="133"/>
-      <c r="D2" s="133"/>
-      <c r="E2" s="133"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="133"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="134"/>
-      <c r="J2" s="134"/>
-      <c r="K2" s="134"/>
-      <c r="L2" s="134"/>
-      <c r="M2" s="134"/>
-      <c r="N2" s="134"/>
-      <c r="O2" s="135"/>
-      <c r="P2" s="136"/>
-      <c r="Q2" s="136"/>
-      <c r="R2" s="136"/>
-      <c r="S2" s="136"/>
-      <c r="T2" s="136"/>
+      <c r="C2" s="138"/>
+      <c r="D2" s="138"/>
+      <c r="E2" s="138"/>
+      <c r="F2" s="138"/>
+      <c r="G2" s="138"/>
+      <c r="H2" s="138"/>
+      <c r="I2" s="139"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="139"/>
+      <c r="L2" s="139"/>
+      <c r="M2" s="139"/>
+      <c r="N2" s="139"/>
+      <c r="O2" s="140"/>
+      <c r="P2" s="141"/>
+      <c r="Q2" s="141"/>
+      <c r="R2" s="141"/>
+      <c r="S2" s="141"/>
+      <c r="T2" s="141"/>
       <c r="U2" s="18"/>
       <c r="V2" s="18"/>
       <c r="W2" s="18"/>
@@ -10775,7 +10774,7 @@
       </c>
       <c r="C6" s="32" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Hitos435[Inicio])=0,TODAY(),B11(Hitos435[Inicio])),TODAY())</f>
-        <v>46133</v>
+        <v>46141</v>
       </c>
       <c r="D6" s="122"/>
       <c r="E6" s="30"/>
@@ -10794,7 +10793,7 @@
       <c r="O6" s="86"/>
       <c r="P6" s="86" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>mayo</v>
       </c>
       <c r="Q6" s="86"/>
       <c r="R6" s="86"/>
@@ -10804,7 +10803,7 @@
       <c r="V6" s="86"/>
       <c r="W6" s="86" t="str">
         <f ca="1">IF(OR(TEXT(W7,"mmmm")=P6,TEXT(W7,"mmmm")=I6),"",TEXT(W7,"mmmm"))</f>
-        <v>mayo</v>
+        <v/>
       </c>
       <c r="X6" s="86"/>
       <c r="Y6" s="86"/>
@@ -10834,7 +10833,7 @@
       <c r="AQ6" s="86"/>
       <c r="AR6" s="86" t="str">
         <f ca="1">IF(OR(TEXT(AR7,"mmmm")=AK6,TEXT(AR7,"mmmm")=AD6,TEXT(AR7,"mmmm")=W6,TEXT(AR7,"mmmm")=P6),"",TEXT(AR7,"mmmm"))</f>
-        <v/>
+        <v>junio</v>
       </c>
       <c r="AS6" s="86"/>
       <c r="AT6" s="86"/>
@@ -10844,7 +10843,7 @@
       <c r="AX6" s="86"/>
       <c r="AY6" s="86" t="str">
         <f ca="1">IF(OR(TEXT(AY7,"mmmm")=AR6,TEXT(AY7,"mmmm")=AK6,TEXT(AY7,"mmmm")=AD6,TEXT(AY7,"mmmm")=W6),"",TEXT(AY7,"mmmm"))</f>
-        <v>junio</v>
+        <v/>
       </c>
       <c r="AZ6" s="86"/>
       <c r="BA6" s="86"/>
@@ -10879,227 +10878,227 @@
       <c r="H7" s="27"/>
       <c r="I7" s="115">
         <f ca="1">IFERROR(Inicio_del_proyecto+Incremento_de_desplazamiento,TODAY())</f>
-        <v>46134</v>
+        <v>46142</v>
       </c>
       <c r="J7" s="116">
         <f ca="1">I7+1</f>
-        <v>46135</v>
+        <v>46143</v>
       </c>
       <c r="K7" s="116">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46136</v>
+        <v>46144</v>
       </c>
       <c r="L7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46137</v>
+        <v>46145</v>
       </c>
       <c r="M7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46138</v>
+        <v>46146</v>
       </c>
       <c r="N7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="O7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="P7" s="116">
         <f ca="1">O7+1</f>
-        <v>46141</v>
+        <v>46149</v>
       </c>
       <c r="Q7" s="116">
         <f ca="1">P7+1</f>
-        <v>46142</v>
+        <v>46150</v>
       </c>
       <c r="R7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46143</v>
+        <v>46151</v>
       </c>
       <c r="S7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46144</v>
+        <v>46152</v>
       </c>
       <c r="T7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46145</v>
+        <v>46153</v>
       </c>
       <c r="U7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="V7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46147</v>
+        <v>46155</v>
       </c>
       <c r="W7" s="116">
         <f ca="1">V7+1</f>
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="X7" s="116">
         <f ca="1">W7+1</f>
-        <v>46149</v>
+        <v>46157</v>
       </c>
       <c r="Y7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46150</v>
+        <v>46158</v>
       </c>
       <c r="Z7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46151</v>
+        <v>46159</v>
       </c>
       <c r="AA7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46152</v>
+        <v>46160</v>
       </c>
       <c r="AB7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46153</v>
+        <v>46161</v>
       </c>
       <c r="AC7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46154</v>
+        <v>46162</v>
       </c>
       <c r="AD7" s="116">
         <f ca="1">AC7+1</f>
-        <v>46155</v>
+        <v>46163</v>
       </c>
       <c r="AE7" s="116">
         <f ca="1">AD7+1</f>
-        <v>46156</v>
+        <v>46164</v>
       </c>
       <c r="AF7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46157</v>
+        <v>46165</v>
       </c>
       <c r="AG7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46158</v>
+        <v>46166</v>
       </c>
       <c r="AH7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46159</v>
+        <v>46167</v>
       </c>
       <c r="AI7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46160</v>
+        <v>46168</v>
       </c>
       <c r="AJ7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46161</v>
+        <v>46169</v>
       </c>
       <c r="AK7" s="116">
         <f ca="1">AJ7+1</f>
-        <v>46162</v>
+        <v>46170</v>
       </c>
       <c r="AL7" s="116">
         <f ca="1">AK7+1</f>
-        <v>46163</v>
+        <v>46171</v>
       </c>
       <c r="AM7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46164</v>
+        <v>46172</v>
       </c>
       <c r="AN7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46165</v>
+        <v>46173</v>
       </c>
       <c r="AO7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46166</v>
+        <v>46174</v>
       </c>
       <c r="AP7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46167</v>
+        <v>46175</v>
       </c>
       <c r="AQ7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46168</v>
+        <v>46176</v>
       </c>
       <c r="AR7" s="116">
         <f ca="1">AQ7+1</f>
-        <v>46169</v>
+        <v>46177</v>
       </c>
       <c r="AS7" s="116">
         <f ca="1">AR7+1</f>
-        <v>46170</v>
+        <v>46178</v>
       </c>
       <c r="AT7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46171</v>
+        <v>46179</v>
       </c>
       <c r="AU7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46172</v>
+        <v>46180</v>
       </c>
       <c r="AV7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46173</v>
+        <v>46181</v>
       </c>
       <c r="AW7" s="116">
         <f t="shared" ca="1" si="0"/>
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="AX7" s="117">
         <f t="shared" ca="1" si="0"/>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AY7" s="116">
         <f ca="1">AX7+1</f>
-        <v>46176</v>
+        <v>46184</v>
       </c>
       <c r="AZ7" s="116">
         <f ca="1">AY7+1</f>
-        <v>46177</v>
+        <v>46185</v>
       </c>
       <c r="BA7" s="116">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46178</v>
+        <v>46186</v>
       </c>
       <c r="BB7" s="116">
         <f t="shared" ca="1" si="1"/>
-        <v>46179</v>
+        <v>46187</v>
       </c>
       <c r="BC7" s="116">
         <f t="shared" ca="1" si="1"/>
-        <v>46180</v>
+        <v>46188</v>
       </c>
       <c r="BD7" s="116">
         <f t="shared" ca="1" si="1"/>
-        <v>46181</v>
+        <v>46189</v>
       </c>
       <c r="BE7" s="117">
         <f t="shared" ca="1" si="1"/>
-        <v>46182</v>
+        <v>46190</v>
       </c>
       <c r="BF7" s="116">
         <f ca="1">BE7+1</f>
-        <v>46183</v>
+        <v>46191</v>
       </c>
       <c r="BG7" s="116">
         <f ca="1">BF7+1</f>
-        <v>46184</v>
+        <v>46192</v>
       </c>
       <c r="BH7" s="116">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46185</v>
+        <v>46193</v>
       </c>
       <c r="BI7" s="116">
         <f t="shared" ca="1" si="2"/>
-        <v>46186</v>
+        <v>46194</v>
       </c>
       <c r="BJ7" s="116">
         <f t="shared" ca="1" si="2"/>
-        <v>46187</v>
+        <v>46195</v>
       </c>
       <c r="BK7" s="116">
         <f t="shared" ca="1" si="2"/>
-        <v>46188</v>
+        <v>46196</v>
       </c>
       <c r="BL7" s="118">
         <f t="shared" ca="1" si="2"/>
-        <v>46189</v>
+        <v>46197</v>
       </c>
       <c r="BM7" s="30"/>
     </row>
@@ -11193,27 +11192,27 @@
       <c r="H9" s="43"/>
       <c r="I9" s="35" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="J9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="K9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="L9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="M9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="N9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="O9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11221,27 +11220,27 @@
       </c>
       <c r="P9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="Q9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="R9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="S9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="T9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="U9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="V9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11249,27 +11248,27 @@
       </c>
       <c r="W9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="X9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="Y9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="Z9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AA9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AB9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AC9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11277,27 +11276,27 @@
       </c>
       <c r="AD9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AE9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AF9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AG9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AH9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AI9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AJ9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11305,27 +11304,27 @@
       </c>
       <c r="AK9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AL9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AM9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AN9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AO9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AP9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AQ9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11333,27 +11332,27 @@
       </c>
       <c r="AR9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AS9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AT9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AU9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AV9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AW9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AX9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11361,27 +11360,27 @@
       </c>
       <c r="AY9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AZ9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="BA9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="BB9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="BC9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="BD9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="BE9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11389,27 +11388,27 @@
       </c>
       <c r="BF9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="BG9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="BH9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="BI9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="BJ9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="BK9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="BL9" s="35" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11737,7 +11736,7 @@
       </c>
       <c r="F12" s="21">
         <f ca="1">TODAY()</f>
-        <v>46133</v>
+        <v>46141</v>
       </c>
       <c r="G12" s="22">
         <v>3</v>
@@ -11981,7 +11980,7 @@
       <c r="E13" s="20"/>
       <c r="F13" s="21">
         <f ca="1">TODAY()+5</f>
-        <v>46138</v>
+        <v>46146</v>
       </c>
       <c r="G13" s="22">
         <v>1</v>
@@ -12227,7 +12226,7 @@
       </c>
       <c r="F14" s="21">
         <f ca="1">F12-3</f>
-        <v>46130</v>
+        <v>46138</v>
       </c>
       <c r="G14" s="22">
         <v>10</v>
@@ -12471,7 +12470,7 @@
       <c r="E15" s="20"/>
       <c r="F15" s="21">
         <f ca="1">F12+20</f>
-        <v>46153</v>
+        <v>46161</v>
       </c>
       <c r="G15" s="22">
         <v>1</v>
@@ -12717,7 +12716,7 @@
       </c>
       <c r="F16" s="21">
         <f ca="1">F12+6</f>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="G16" s="22">
         <v>6</v>
@@ -13200,7 +13199,7 @@
       </c>
       <c r="F18" s="21">
         <f ca="1">F12+6</f>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="G18" s="22">
         <v>13</v>
@@ -13446,7 +13445,7 @@
       </c>
       <c r="F19" s="21">
         <f ca="1">F18+2</f>
-        <v>46141</v>
+        <v>46149</v>
       </c>
       <c r="G19" s="22">
         <v>9</v>
@@ -13692,7 +13691,7 @@
       </c>
       <c r="F20" s="21">
         <f ca="1">F19+5</f>
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="G20" s="22">
         <v>11</v>
@@ -13936,7 +13935,7 @@
       <c r="E21" s="20"/>
       <c r="F21" s="21">
         <f ca="1">F20+2</f>
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="G21" s="22">
         <v>1</v>
@@ -14178,7 +14177,7 @@
       <c r="E22" s="20"/>
       <c r="F22" s="21">
         <f ca="1">F21+1</f>
-        <v>46149</v>
+        <v>46157</v>
       </c>
       <c r="G22" s="22">
         <v>24</v>
@@ -14659,7 +14658,7 @@
       <c r="E24" s="20"/>
       <c r="F24" s="21">
         <f ca="1">F12+15</f>
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="G24" s="22">
         <v>4</v>
@@ -14903,7 +14902,7 @@
       <c r="E25" s="20"/>
       <c r="F25" s="21">
         <f ca="1">F24+3</f>
-        <v>46151</v>
+        <v>46159</v>
       </c>
       <c r="G25" s="22">
         <v>14</v>
@@ -15147,7 +15146,7 @@
       <c r="E26" s="20"/>
       <c r="F26" s="21">
         <f ca="1">F25+15</f>
-        <v>46166</v>
+        <v>46174</v>
       </c>
       <c r="G26" s="22">
         <v>6</v>
@@ -15391,7 +15390,7 @@
       <c r="E27" s="20"/>
       <c r="F27" s="21">
         <f ca="1">F21+22</f>
-        <v>46170</v>
+        <v>46178</v>
       </c>
       <c r="G27" s="22">
         <v>3</v>
@@ -15635,7 +15634,7 @@
       <c r="E28" s="20"/>
       <c r="F28" s="21">
         <f ca="1">F16</f>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="G28" s="22">
         <v>19</v>
@@ -16114,7 +16113,7 @@
       <c r="E30" s="20"/>
       <c r="F30" s="21">
         <f ca="1">F27+3</f>
-        <v>46173</v>
+        <v>46181</v>
       </c>
       <c r="G30" s="22">
         <v>15</v>
@@ -16356,7 +16355,7 @@
       <c r="E31" s="20"/>
       <c r="F31" s="21">
         <f ca="1">F30+14</f>
-        <v>46187</v>
+        <v>46195</v>
       </c>
       <c r="G31" s="22">
         <v>5</v>
@@ -16600,7 +16599,7 @@
       <c r="E32" s="20"/>
       <c r="F32" s="21">
         <f ca="1">F31+42</f>
-        <v>46229</v>
+        <v>46237</v>
       </c>
       <c r="G32" s="22">
         <v>1</v>
@@ -17820,27 +17819,27 @@
     <row r="1" spans="1:68" ht="25.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:68" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10"/>
-      <c r="B2" s="137" t="s">
+      <c r="B2" s="127" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="137"/>
-      <c r="D2" s="137"/>
-      <c r="E2" s="137"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="137"/>
-      <c r="H2" s="137"/>
-      <c r="I2" s="138"/>
-      <c r="J2" s="138"/>
-      <c r="K2" s="138"/>
-      <c r="L2" s="138"/>
-      <c r="M2" s="138"/>
-      <c r="N2" s="138"/>
-      <c r="O2" s="139"/>
-      <c r="P2" s="139"/>
-      <c r="Q2" s="139"/>
-      <c r="R2" s="139"/>
-      <c r="S2" s="139"/>
-      <c r="T2" s="139"/>
+      <c r="C2" s="127"/>
+      <c r="D2" s="127"/>
+      <c r="E2" s="127"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="127"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="128"/>
+      <c r="J2" s="128"/>
+      <c r="K2" s="128"/>
+      <c r="L2" s="128"/>
+      <c r="M2" s="128"/>
+      <c r="N2" s="128"/>
+      <c r="O2" s="129"/>
+      <c r="P2" s="129"/>
+      <c r="Q2" s="129"/>
+      <c r="R2" s="129"/>
+      <c r="S2" s="129"/>
+      <c r="T2" s="129"/>
       <c r="U2" s="88"/>
       <c r="V2" s="88"/>
       <c r="W2" s="88"/>
@@ -17962,9 +17961,9 @@
       <c r="B6" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="140" cm="1">
+      <c r="C6" s="73" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Hitos43524[Inicio])=0,TODAY(),B11(Hitos43524[Inicio])),TODAY())-35</f>
-        <v>46098</v>
+        <v>46106</v>
       </c>
       <c r="D6" s="73"/>
       <c r="E6" s="68"/>
@@ -17983,7 +17982,7 @@
       <c r="O6" s="83"/>
       <c r="P6" s="83" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>abril</v>
       </c>
       <c r="Q6" s="83"/>
       <c r="R6" s="83"/>
@@ -18003,7 +18002,7 @@
       <c r="AC6" s="83"/>
       <c r="AD6" s="83" t="str">
         <f ca="1">IF(OR(TEXT(AD7,"mmmm")=W6,TEXT(AD7,"mmmm")=P6,TEXT(AD7,"mmmm")=I6),"",TEXT(AD7,"mmmm"))</f>
-        <v>abril</v>
+        <v/>
       </c>
       <c r="AE6" s="83"/>
       <c r="AF6" s="83"/>
@@ -18033,7 +18032,7 @@
       <c r="AX6" s="84"/>
       <c r="AY6" s="84" t="str">
         <f ca="1">IF(OR(TEXT(AY7,"mmmm")=AR6,TEXT(AY7,"mmmm")=AK6,TEXT(AY7,"mmmm")=AD6,TEXT(AY7,"mmmm")=W6),"",TEXT(AY7,"mmmm"))</f>
-        <v/>
+        <v>mayo</v>
       </c>
       <c r="AZ6" s="84"/>
       <c r="BA6" s="84"/>
@@ -18043,7 +18042,7 @@
       <c r="BE6" s="82"/>
       <c r="BF6" s="82" t="str">
         <f ca="1">IF(OR(TEXT(BF7,"mmmm")=AY6,TEXT(BF7,"mmmm")=AR6,TEXT(BF7,"mmmm")=AK6,TEXT(BF7,"mmmm")=AD6),"",TEXT(BF7,"mmmm"))</f>
-        <v>mayo</v>
+        <v/>
       </c>
       <c r="BG6" s="82"/>
       <c r="BH6" s="82"/>
@@ -18067,227 +18066,227 @@
       <c r="H7" s="75"/>
       <c r="I7" s="107">
         <f ca="1">IFERROR(Inicio_del_proyecto+Incremento_de_desplazamiento,TODAY())</f>
-        <v>46098</v>
+        <v>46106</v>
       </c>
       <c r="J7" s="108">
         <f ca="1">I7+1</f>
-        <v>46099</v>
+        <v>46107</v>
       </c>
       <c r="K7" s="108">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46100</v>
+        <v>46108</v>
       </c>
       <c r="L7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46101</v>
+        <v>46109</v>
       </c>
       <c r="M7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46102</v>
+        <v>46110</v>
       </c>
       <c r="N7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46103</v>
+        <v>46111</v>
       </c>
       <c r="O7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46104</v>
+        <v>46112</v>
       </c>
       <c r="P7" s="108">
         <f ca="1">O7+1</f>
-        <v>46105</v>
+        <v>46113</v>
       </c>
       <c r="Q7" s="108">
         <f ca="1">P7+1</f>
-        <v>46106</v>
+        <v>46114</v>
       </c>
       <c r="R7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46107</v>
+        <v>46115</v>
       </c>
       <c r="S7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46108</v>
+        <v>46116</v>
       </c>
       <c r="T7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46109</v>
+        <v>46117</v>
       </c>
       <c r="U7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46110</v>
+        <v>46118</v>
       </c>
       <c r="V7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46111</v>
+        <v>46119</v>
       </c>
       <c r="W7" s="108">
         <f ca="1">V7+1</f>
-        <v>46112</v>
+        <v>46120</v>
       </c>
       <c r="X7" s="108">
         <f ca="1">W7+1</f>
-        <v>46113</v>
+        <v>46121</v>
       </c>
       <c r="Y7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46114</v>
+        <v>46122</v>
       </c>
       <c r="Z7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46115</v>
+        <v>46123</v>
       </c>
       <c r="AA7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46116</v>
+        <v>46124</v>
       </c>
       <c r="AB7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46117</v>
+        <v>46125</v>
       </c>
       <c r="AC7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46118</v>
+        <v>46126</v>
       </c>
       <c r="AD7" s="108">
         <f ca="1">AC7+1</f>
-        <v>46119</v>
+        <v>46127</v>
       </c>
       <c r="AE7" s="108">
         <f ca="1">AD7+1</f>
-        <v>46120</v>
+        <v>46128</v>
       </c>
       <c r="AF7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46121</v>
+        <v>46129</v>
       </c>
       <c r="AG7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46122</v>
+        <v>46130</v>
       </c>
       <c r="AH7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46123</v>
+        <v>46131</v>
       </c>
       <c r="AI7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46124</v>
+        <v>46132</v>
       </c>
       <c r="AJ7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46125</v>
+        <v>46133</v>
       </c>
       <c r="AK7" s="108">
         <f ca="1">AJ7+1</f>
-        <v>46126</v>
+        <v>46134</v>
       </c>
       <c r="AL7" s="108">
         <f ca="1">AK7+1</f>
-        <v>46127</v>
+        <v>46135</v>
       </c>
       <c r="AM7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46128</v>
+        <v>46136</v>
       </c>
       <c r="AN7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46129</v>
+        <v>46137</v>
       </c>
       <c r="AO7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46130</v>
+        <v>46138</v>
       </c>
       <c r="AP7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46131</v>
+        <v>46139</v>
       </c>
       <c r="AQ7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46132</v>
+        <v>46140</v>
       </c>
       <c r="AR7" s="108">
         <f ca="1">AQ7+1</f>
-        <v>46133</v>
+        <v>46141</v>
       </c>
       <c r="AS7" s="108">
         <f ca="1">AR7+1</f>
-        <v>46134</v>
+        <v>46142</v>
       </c>
       <c r="AT7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46135</v>
+        <v>46143</v>
       </c>
       <c r="AU7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46136</v>
+        <v>46144</v>
       </c>
       <c r="AV7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46137</v>
+        <v>46145</v>
       </c>
       <c r="AW7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46138</v>
+        <v>46146</v>
       </c>
       <c r="AX7" s="109">
         <f t="shared" ca="1" si="0"/>
-        <v>46139</v>
+        <v>46147</v>
       </c>
       <c r="AY7" s="108">
         <f ca="1">AX7+1</f>
-        <v>46140</v>
+        <v>46148</v>
       </c>
       <c r="AZ7" s="108">
         <f ca="1">AY7+1</f>
-        <v>46141</v>
+        <v>46149</v>
       </c>
       <c r="BA7" s="108">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46142</v>
+        <v>46150</v>
       </c>
       <c r="BB7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46143</v>
+        <v>46151</v>
       </c>
       <c r="BC7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46144</v>
+        <v>46152</v>
       </c>
       <c r="BD7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46145</v>
+        <v>46153</v>
       </c>
       <c r="BE7" s="109">
         <f t="shared" ca="1" si="1"/>
-        <v>46146</v>
+        <v>46154</v>
       </c>
       <c r="BF7" s="108">
         <f ca="1">BE7+1</f>
-        <v>46147</v>
+        <v>46155</v>
       </c>
       <c r="BG7" s="108">
         <f ca="1">BF7+1</f>
-        <v>46148</v>
+        <v>46156</v>
       </c>
       <c r="BH7" s="108">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46149</v>
+        <v>46157</v>
       </c>
       <c r="BI7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46150</v>
+        <v>46158</v>
       </c>
       <c r="BJ7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46151</v>
+        <v>46159</v>
       </c>
       <c r="BK7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46152</v>
+        <v>46160</v>
       </c>
       <c r="BL7" s="109">
         <f t="shared" ca="1" si="2"/>
-        <v>46153</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -18383,27 +18382,27 @@
       </c>
       <c r="J9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="K9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="L9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="M9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="N9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="O9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="P9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18411,27 +18410,27 @@
       </c>
       <c r="Q9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="R9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="S9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="T9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="U9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="V9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="W9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18439,27 +18438,27 @@
       </c>
       <c r="X9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="Y9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="Z9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AA9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AB9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AC9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AD9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18467,27 +18466,27 @@
       </c>
       <c r="AE9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AF9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AG9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AH9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AI9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AJ9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AK9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18495,27 +18494,27 @@
       </c>
       <c r="AL9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AM9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AN9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AO9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AP9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AQ9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AR9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18523,27 +18522,27 @@
       </c>
       <c r="AS9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="AT9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="AU9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="AV9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AW9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="AX9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="AY9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18551,27 +18550,27 @@
       </c>
       <c r="AZ9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="BA9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="BB9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="BC9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="BD9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="BE9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
       <c r="BF9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18579,27 +18578,27 @@
       </c>
       <c r="BG9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>m</v>
+        <v>j</v>
       </c>
       <c r="BH9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>j</v>
+        <v>v</v>
       </c>
       <c r="BI9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>v</v>
+        <v>s</v>
       </c>
       <c r="BJ9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="BK9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>l</v>
       </c>
       <c r="BL9" s="89" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>l</v>
+        <v>m</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -18609,7 +18608,7 @@
       <c r="E10" s="13"/>
       <c r="F10" s="14">
         <f t="shared" ref="F10:F12" ca="1" si="4">TODAY()-35</f>
-        <v>46098</v>
+        <v>46106</v>
       </c>
       <c r="G10" s="15"/>
       <c r="I10" s="34"/>
@@ -18922,7 +18921,7 @@
       </c>
       <c r="F12" s="55">
         <f t="shared" ca="1" si="4"/>
-        <v>46098</v>
+        <v>46106</v>
       </c>
       <c r="G12" s="56">
         <v>1</v>
@@ -19163,7 +19162,7 @@
       <c r="E13" s="54"/>
       <c r="F13" s="55">
         <f ca="1">TODAY()-35</f>
-        <v>46098</v>
+        <v>46106</v>
       </c>
       <c r="G13" s="56">
         <v>1</v>
@@ -19408,7 +19407,7 @@
       </c>
       <c r="F14" s="55">
         <f ca="1">TODAY()-34</f>
-        <v>46099</v>
+        <v>46107</v>
       </c>
       <c r="G14" s="56">
         <v>4</v>
@@ -19649,7 +19648,7 @@
       <c r="E15" s="54"/>
       <c r="F15" s="55">
         <f ca="1">TODAY()-34</f>
-        <v>46099</v>
+        <v>46107</v>
       </c>
       <c r="G15" s="56">
         <v>4</v>
@@ -19894,7 +19893,7 @@
       </c>
       <c r="F16" s="55">
         <f ca="1">TODAY()-30</f>
-        <v>46103</v>
+        <v>46111</v>
       </c>
       <c r="G16" s="56">
         <v>4</v>
@@ -20127,7 +20126,7 @@
     </row>
     <row r="17" spans="1:64" s="1" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9"/>
-      <c r="B17" s="141"/>
+      <c r="B17" s="123"/>
       <c r="C17" s="53" t="s">
         <v>21</v>
       </c>
@@ -20135,7 +20134,7 @@
       <c r="E17" s="54"/>
       <c r="F17" s="55">
         <f ca="1">TODAY()-30</f>
-        <v>46103</v>
+        <v>46111</v>
       </c>
       <c r="G17" s="56">
         <v>4</v>
@@ -20460,7 +20459,7 @@
       </c>
       <c r="F19" s="55">
         <f ca="1">TODAY()-20</f>
-        <v>46113</v>
+        <v>46121</v>
       </c>
       <c r="G19" s="56">
         <v>13</v>
@@ -20701,11 +20700,11 @@
       </c>
       <c r="D20" s="53"/>
       <c r="E20" s="54">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="F20" s="55">
         <f ca="1">TODAY()+2</f>
-        <v>46135</v>
+        <v>46143</v>
       </c>
       <c r="G20" s="56">
         <v>9</v>
@@ -20945,12 +20944,12 @@
         <v>23</v>
       </c>
       <c r="D21" s="53"/>
-      <c r="E21" s="54">
+      <c r="E21" s="142">
         <v>0</v>
       </c>
       <c r="F21" s="55">
         <f ca="1">TODAY()+5</f>
-        <v>46138</v>
+        <v>46146</v>
       </c>
       <c r="G21" s="56">
         <v>11</v>
@@ -21191,7 +21190,7 @@
       <c r="E22" s="54"/>
       <c r="F22" s="55">
         <f ca="1">TODAY()+10</f>
-        <v>46143</v>
+        <v>46151</v>
       </c>
       <c r="G22" s="56">
         <v>10</v>
@@ -21432,234 +21431,234 @@
       <c r="G23" s="56"/>
       <c r="H23" s="53"/>
       <c r="I23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ref="I23:AN23" ca="1" si="11">IF(AND($C23="Objetivo",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1),1,""))</f>
         <v/>
       </c>
       <c r="J23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",J$7&gt;=$F23,J$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",J$7&gt;=$F23,J$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="K23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",K$7&gt;=$F23,K$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",K$7&gt;=$F23,K$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="L23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",L$7&gt;=$F23,L$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",L$7&gt;=$F23,L$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="M23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",M$7&gt;=$F23,M$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",M$7&gt;=$F23,M$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="N23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",N$7&gt;=$F23,N$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",N$7&gt;=$F23,N$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="O23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",O$7&gt;=$F23,O$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",O$7&gt;=$F23,O$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="P23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",P$7&gt;=$F23,P$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",P$7&gt;=$F23,P$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="Q23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",Q$7&gt;=$F23,Q$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",Q$7&gt;=$F23,Q$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="R23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",R$7&gt;=$F23,R$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",R$7&gt;=$F23,R$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",S$7&gt;=$F23,S$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",S$7&gt;=$F23,S$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="T23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",T$7&gt;=$F23,T$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",T$7&gt;=$F23,T$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="U23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",U$7&gt;=$F23,U$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",U$7&gt;=$F23,U$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="V23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",V$7&gt;=$F23,V$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",V$7&gt;=$F23,V$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="W23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",W$7&gt;=$F23,W$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",W$7&gt;=$F23,W$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="X23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",X$7&gt;=$F23,X$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",X$7&gt;=$F23,X$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="Y23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",Y$7&gt;=$F23,Y$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",Y$7&gt;=$F23,Y$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="Z23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",Z$7&gt;=$F23,Z$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",Z$7&gt;=$F23,Z$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AA23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AA$7&gt;=$F23,AA$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AA$7&gt;=$F23,AA$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AB23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AB$7&gt;=$F23,AB$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AB$7&gt;=$F23,AB$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AC23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AC$7&gt;=$F23,AC$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AC$7&gt;=$F23,AC$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AD23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AD$7&gt;=$F23,AD$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AD$7&gt;=$F23,AD$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AE23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AE$7&gt;=$F23,AE$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AE$7&gt;=$F23,AE$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AF23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AF$7&gt;=$F23,AF$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AF$7&gt;=$F23,AF$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AG23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AG$7&gt;=$F23,AG$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AG$7&gt;=$F23,AG$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AH23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AH$7&gt;=$F23,AH$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AH$7&gt;=$F23,AH$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AI23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AI$7&gt;=$F23,AI$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AI$7&gt;=$F23,AI$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AJ23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AJ$7&gt;=$F23,AJ$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AJ$7&gt;=$F23,AJ$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AK23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AK$7&gt;=$F23,AK$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AK$7&gt;=$F23,AK$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AL23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AL$7&gt;=$F23,AL$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AL$7&gt;=$F23,AL$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AM23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AM$7&gt;=$F23,AM$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AM$7&gt;=$F23,AM$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AN23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AN$7&gt;=$F23,AN$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AN$7&gt;=$F23,AN$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="AO23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AO$7&gt;=$F23,AO$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AO$7&gt;=$F23,AO$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ref="AO23:BL23" ca="1" si="12">IF(AND($C23="Objetivo",AO$7&gt;=$F23,AO$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AO$7&gt;=$F23,AO$7&lt;=$F23+$G23-1),1,""))</f>
         <v/>
       </c>
       <c r="AP23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AP$7&gt;=$F23,AP$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AP$7&gt;=$F23,AP$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AQ23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AQ$7&gt;=$F23,AQ$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AQ$7&gt;=$F23,AQ$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AR23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AR$7&gt;=$F23,AR$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AR$7&gt;=$F23,AR$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AS23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AS$7&gt;=$F23,AS$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AS$7&gt;=$F23,AS$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AT23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AT$7&gt;=$F23,AT$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AT$7&gt;=$F23,AT$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AU23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AU$7&gt;=$F23,AU$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AU$7&gt;=$F23,AU$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AV23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AV$7&gt;=$F23,AV$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AV$7&gt;=$F23,AV$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AW23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AW$7&gt;=$F23,AW$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AW$7&gt;=$F23,AW$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AX23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AX$7&gt;=$F23,AX$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AX$7&gt;=$F23,AX$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AY23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AY$7&gt;=$F23,AY$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AY$7&gt;=$F23,AY$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="AZ23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",AZ$7&gt;=$F23,AZ$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",AZ$7&gt;=$F23,AZ$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BA23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BA$7&gt;=$F23,BA$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BA$7&gt;=$F23,BA$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BB23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BB$7&gt;=$F23,BB$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BB$7&gt;=$F23,BB$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BC23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BC$7&gt;=$F23,BC$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BC$7&gt;=$F23,BC$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BD23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BD$7&gt;=$F23,BD$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BD$7&gt;=$F23,BD$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BE23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BE$7&gt;=$F23,BE$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BE$7&gt;=$F23,BE$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BF23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BF$7&gt;=$F23,BF$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BF$7&gt;=$F23,BF$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BG23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BG$7&gt;=$F23,BG$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BG$7&gt;=$F23,BG$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BH23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BH$7&gt;=$F23,BH$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BH$7&gt;=$F23,BH$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BI23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BI$7&gt;=$F23,BI$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BI$7&gt;=$F23,BI$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BJ23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BJ$7&gt;=$F23,BJ$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BJ$7&gt;=$F23,BJ$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BK23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BK$7&gt;=$F23,BK$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BK$7&gt;=$F23,BK$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
       <c r="BL23" s="24" t="str">
-        <f ca="1">IF(AND($C23="Objetivo",BL$7&gt;=$F23,BL$7&lt;=$F23+$G23-1),2,IF(AND($C23="Hito",BL$7&gt;=$F23,BL$7&lt;=$F23+$G23-1),1,""))</f>
+        <f t="shared" ca="1" si="12"/>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:64" s="1" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9"/>
       <c r="B24"/>
-      <c r="C24" s="142"/>
+      <c r="C24" s="124"/>
       <c r="D24" s="4"/>
       <c r="E24"/>
       <c r="F24" s="2"/>
@@ -22304,26 +22303,26 @@
       <formula>AND(LEN($C10)=0,I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J6:BL6">
-    <cfRule type="expression" dxfId="5" priority="3">
-      <formula>AND(J$7&lt;=EOMONTH($I$7,2),J$7&gt;EOMONTH($I$7,0),J$7&gt;EOMONTH($I$7,1))</formula>
+  <conditionalFormatting sqref="I23:BL23">
+    <cfRule type="expression" dxfId="5" priority="22" stopIfTrue="1">
+      <formula>AND($C23="Riesgo bajo",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="23" stopIfTrue="1">
+      <formula>AND($C23="Riesgo alto",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="24" stopIfTrue="1">
+      <formula>AND($C23="Según lo previsto",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="25" stopIfTrue="1">
+      <formula>AND($C23="Riesgo medio",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="26" stopIfTrue="1">
+      <formula>AND(LEN($C23)=0,I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I23:BL23">
-    <cfRule type="expression" dxfId="4" priority="22" stopIfTrue="1">
-      <formula>AND($C23="Riesgo bajo",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="23" stopIfTrue="1">
-      <formula>AND($C23="Riesgo alto",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="24" stopIfTrue="1">
-      <formula>AND($C23="Según lo previsto",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="25" stopIfTrue="1">
-      <formula>AND($C23="Riesgo medio",I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="26" stopIfTrue="1">
-      <formula>AND(LEN($C23)=0,I$7&gt;=$F23,I$7&lt;=$F23+$G23-1)</formula>
+  <conditionalFormatting sqref="J6:BL6">
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>AND(J$7&lt;=EOMONTH($I$7,2),J$7&gt;EOMONTH($I$7,0),J$7&gt;EOMONTH($I$7,1))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="13">
@@ -22420,6 +22419,25 @@
           <xm:sqref>I10:BL22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="iconSet" priority="21" id="{67763332-2AE9-4F93-8BB7-5ECDB6B99BA2}">
+            <x14:iconSet iconSet="3Stars" showValue="0" custom="1">
+              <x14:cfvo type="percent">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:cfIcon iconSet="NoIcons" iconId="0"/>
+              <x14:cfIcon iconSet="3Flags" iconId="1"/>
+              <x14:cfIcon iconSet="3Signs" iconId="0"/>
+            </x14:iconSet>
+          </x14:cfRule>
+          <xm:sqref>I23:BL23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="iconSet" priority="12" id="{5AD67FB9-23B4-4F54-BD80-7A6CF9720346}">
             <x14:iconSet iconSet="3Stars" showValue="0" custom="1">
               <x14:cfvo type="percent">
@@ -22437,25 +22455,6 @@
             </x14:iconSet>
           </x14:cfRule>
           <xm:sqref>I30:BL30</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="iconSet" priority="21" id="{67763332-2AE9-4F93-8BB7-5ECDB6B99BA2}">
-            <x14:iconSet iconSet="3Stars" showValue="0" custom="1">
-              <x14:cfvo type="percent">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:cfIcon iconSet="NoIcons" iconId="0"/>
-              <x14:cfIcon iconSet="3Flags" iconId="1"/>
-              <x14:cfIcon iconSet="3Signs" iconId="0"/>
-            </x14:iconSet>
-          </x14:cfRule>
-          <xm:sqref>I23:BL23</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -22740,15 +22739,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -22765,6 +22755,15 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -22789,14 +22788,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -22806,4 +22797,12 @@
     <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>